<commit_message>
Update editable MCA guidelines workbook
</commit_message>
<xml_diff>
--- a/gokapital-mca-program-guidelines.xlsx
+++ b/gokapital-mca-program-guidelines.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCA Guidelines EN" sheetId="1" r:id="R5535c935adc54c99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guia MCA ES" sheetId="2" r:id="R11fff2105d9c4a5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MCA Guidelines EN" sheetId="1" r:id="R0b97d8a8e5bd4d8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guia MCA ES" sheetId="2" r:id="R5a5c5abc4f054cd1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,7 +14,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="8">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -52,6 +52,12 @@
       <x:b/>
       <x:sz val="11"/>
       <x:color rgb="FF2E8B3A"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF16365D"/>
       <x:name val="Aptos"/>
     </x:font>
     <x:font>
@@ -179,7 +185,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="96">
+  <x:cellXfs count="100">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -396,14 +402,24 @@
     <x:xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -415,7 +431,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="GoKapital" id="{C11C9544-CDC4-4B6B-941A-62938801B2E5}"/>
+  <xltc:person displayName="GoKapital" id="{61E94E9B-6F58-49F8-8D2F-FCD274D89EA5}"/>
 </xltc:personList>
 </file>
 
@@ -614,12 +630,12 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="31" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="25" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="25" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="36" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -933,19 +949,19 @@
         <x:v>STATE RESTRICTIONS</x:v>
       </x:c>
       <x:c r="B18" s="70" t="str">
-        <x:v>Most states; TX may use a loan structure; CA/NY often require 4 bank months</x:v>
+        <x:v>Most states; TX may use a loan structure</x:v>
       </x:c>
       <x:c r="C18" s="71" t="str">
         <x:v>Availability varies; TX/VA may require stronger revenue or time in business</x:v>
       </x:c>
       <x:c r="D18" s="72" t="str">
-        <x:v>Some programs exclude VA, CT, UT, ND, AR or TX; verify before submission</x:v>
+        <x:v>Some programs exclude VA, CT, UT, ND, AR or TX</x:v>
       </x:c>
       <x:c r="E18" s="73" t="str">
         <x:v>State and entity restrictions can limit specialty programs</x:v>
       </x:c>
       <x:c r="F18" s="74" t="str">
-        <x:v>Restricted-state exceptions are limited; verify before submission</x:v>
+        <x:v>Restricted-state exceptions are limited</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="76" customHeight="1">
@@ -1033,19 +1049,19 @@
         <x:v>SPECIAL CONSIDERATIONS</x:v>
       </x:c>
       <x:c r="B23" s="70" t="str">
-        <x:v>Best value may include longer terms, flexible payments, lower pricing and early-pay options</x:v>
+        <x:v>Early payment discounts; longer terms; flexible payments</x:v>
       </x:c>
       <x:c r="C23" s="71" t="str">
-        <x:v>Strong files may receive better term, payment frequency, renewal or payoff support</x:v>
+        <x:v>Early payment discounts; renewals; payoff options</x:v>
       </x:c>
       <x:c r="D23" s="72" t="str">
-        <x:v>Higher-risk SICs, satisfied defaults or extra positions may be considered with strong offsets</x:v>
+        <x:v>May help build business credit history; renewal access</x:v>
       </x:c>
       <x:c r="E23" s="73" t="str">
-        <x:v>Starter offers, split payments or added financing may be available with compensating factors</x:v>
+        <x:v>Starter funding; may establish payment history</x:v>
       </x:c>
       <x:c r="F23" s="74" t="str">
-        <x:v>Specialty, starter or consolidation structures only; expect smaller and shorter offers</x:v>
+        <x:v>Starter or consolidation options</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="88" customHeight="1">
@@ -1068,7 +1084,7 @@
         <x:v>Financial-fraud concerns; manipulated documents; stop-payments to funders</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="28" customHeight="1">
+    <x:row r="26" ht="32" customHeight="1">
       <x:c r="A26" s="76" t="str">
         <x:v>POSSIBLE EXCEPTIONS &amp; IMPORTANT POINTS</x:v>
       </x:c>
@@ -1083,7 +1099,7 @@
         <x:v>APPROVAL TERMS</x:v>
       </x:c>
       <x:c r="B27" s="84" t="str">
-        <x:v>FUNDING, RATE AND TERM DEPEND ON THE COMPLETE PROFILE, INCLUDING REVENUE, CREDIT, DEBT, BANK ACTIVITY AND INDUSTRY.</x:v>
+        <x:v>Funding, rate and term depend on the complete profile, including revenue, credit, debt, bank activity and industry.</x:v>
       </x:c>
       <x:c r="C27" s="84"/>
       <x:c r="D27" s="84"/>
@@ -1095,7 +1111,7 @@
         <x:v>HIGH-RISK INDUSTRIES</x:v>
       </x:c>
       <x:c r="B28" s="84" t="str">
-        <x:v>REVIEWED CASE BY CASE; APPROVALS ARE GENERALLY SMALLER, SHORTER AND MORE CONSERVATIVE.</x:v>
+        <x:v>Reviewed case by case; approvals are generally smaller, shorter and more conservative.</x:v>
       </x:c>
       <x:c r="C28" s="84"/>
       <x:c r="D28" s="84"/>
@@ -1107,7 +1123,7 @@
         <x:v>CONSOLIDATION</x:v>
       </x:c>
       <x:c r="B29" s="84" t="str">
-        <x:v>MULTIPLE MCAS ARE ALLOWED. ADDED FUNDING, REFINANCE OR CONSOLIDATION MAY BE AVAILABLE SUBJECT TO AFFORDABILITY.</x:v>
+        <x:v>Multiple MCAs are allowed. Added funding, refinance or consolidation may be available subject to affordability.</x:v>
       </x:c>
       <x:c r="C29" s="84"/>
       <x:c r="D29" s="84"/>
@@ -1119,7 +1135,7 @@
         <x:v>ITIN ELIGIBILITY</x:v>
       </x:c>
       <x:c r="B30" s="84" t="str">
-        <x:v>CASE BY CASE: 12+ MONTHS IN BUSINESS AND MORE THAN $25,000 IN MONTHLY REVENUE.</x:v>
+        <x:v>Case by case: 12+ months in business and more than $25,000 in monthly revenue.</x:v>
       </x:c>
       <x:c r="C30" s="84"/>
       <x:c r="D30" s="84"/>
@@ -1131,88 +1147,118 @@
         <x:v>DOCUMENTS</x:v>
       </x:c>
       <x:c r="B31" s="84" t="str">
-        <x:v>TYPICAL STIPS: ID, VOIDED CHECK, OWNERSHIP PROOF AND BANK VERIFICATION. LARGE DEALS MAY NEED TAX RETURNS OR FINANCIALS.</x:v>
+        <x:v>Typical stips: ID, voided check, ownership proof and bank verification. Large deals may need tax returns or financials.</x:v>
       </x:c>
       <x:c r="C31" s="84"/>
       <x:c r="D31" s="84"/>
       <x:c r="E31" s="84"/>
       <x:c r="F31" s="85"/>
     </x:row>
-    <x:row r="33" ht="28" customHeight="1">
-      <x:c r="A33" s="87" t="str">
+    <x:row r="32" ht="62" customHeight="1">
+      <x:c r="A32" s="83" t="str">
+        <x:v>RESPONSE &amp; FUNDING</x:v>
+      </x:c>
+      <x:c r="B32" s="84" t="str">
+        <x:v>Offers may be available within 24 hours. Same-day funding is possible when required information is received promptly.</x:v>
+      </x:c>
+      <x:c r="C32" s="84"/>
+      <x:c r="D32" s="84"/>
+      <x:c r="E32" s="84"/>
+      <x:c r="F32" s="85"/>
+    </x:row>
+    <x:row r="34" ht="32" customHeight="1">
+      <x:c r="A34" s="87" t="str">
         <x:v>MINIMUM REQUIRED DOCUMENTS</x:v>
       </x:c>
-      <x:c r="B33" s="87"/>
-      <x:c r="C33" s="87"/>
-      <x:c r="D33" s="87"/>
-      <x:c r="E33" s="87"/>
-      <x:c r="F33" s="87"/>
-    </x:row>
-    <x:row r="34" ht="44" customHeight="1">
-      <x:c r="A34" s="91" t="n">
+      <x:c r="B34" s="87"/>
+      <x:c r="C34" s="87"/>
+      <x:c r="D34" s="76" t="str">
+        <x:v>LOAN SUBMISSION PROCESS</x:v>
+      </x:c>
+      <x:c r="E34" s="76"/>
+      <x:c r="F34" s="76"/>
+    </x:row>
+    <x:row r="35" ht="58" customHeight="1">
+      <x:c r="A35" s="91" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B34" s="84" t="str">
+      <x:c r="B35" s="84" t="str">
         <x:v>Signed application</x:v>
       </x:c>
-      <x:c r="C34" s="84"/>
-      <x:c r="D34" s="84"/>
-      <x:c r="E34" s="84"/>
-      <x:c r="F34" s="85"/>
-    </x:row>
-    <x:row r="35" ht="44" customHeight="1">
-      <x:c r="A35" s="91" t="n">
+      <x:c r="C35" s="85"/>
+      <x:c r="D35" s="95" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E35" s="84" t="str">
+        <x:v>Gather the signed application and bank statements</x:v>
+      </x:c>
+      <x:c r="F35" s="85"/>
+    </x:row>
+    <x:row r="36" ht="58" customHeight="1">
+      <x:c r="A36" s="91" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B35" s="84" t="str">
+      <x:c r="B36" s="84" t="str">
         <x:v>Most recent 4-6 months of complete business bank statements</x:v>
       </x:c>
-      <x:c r="C35" s="84"/>
-      <x:c r="D35" s="84"/>
-      <x:c r="E35" s="84"/>
-      <x:c r="F35" s="85"/>
-    </x:row>
-    <x:row r="36" ht="54" customHeight="1">
-      <x:c r="A36" s="91" t="n">
+      <x:c r="C36" s="85"/>
+      <x:c r="D36" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E36" s="84" t="str">
+        <x:v>Email the complete file to deals@gokapital.com</x:v>
+      </x:c>
+      <x:c r="F36" s="85"/>
+    </x:row>
+    <x:row r="37" ht="66" customHeight="1">
+      <x:c r="A37" s="91" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B36" s="84" t="str">
+      <x:c r="B37" s="84" t="str">
         <x:v>Requests above $150,000: tax returns and current Profit &amp; Loss statement</x:v>
       </x:c>
-      <x:c r="C36" s="84"/>
-      <x:c r="D36" s="84"/>
-      <x:c r="E36" s="84"/>
-      <x:c r="F36" s="85"/>
-    </x:row>
-    <x:row r="37" ht="54" customHeight="1">
-      <x:c r="A37" s="91" t="n">
+      <x:c r="C37" s="85"/>
+      <x:c r="D37" s="95" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E37" s="84" t="str">
+        <x:v>Same-day response when received before 1:00 PM</x:v>
+      </x:c>
+      <x:c r="F37" s="85"/>
+    </x:row>
+    <x:row r="38" ht="66" customHeight="1">
+      <x:c r="A38" s="91" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B37" s="84" t="str">
+      <x:c r="B38" s="84" t="str">
         <x:v>Consolidation requests: current balance and payoff details</x:v>
       </x:c>
-      <x:c r="C37" s="84"/>
-      <x:c r="D37" s="84"/>
-      <x:c r="E37" s="84"/>
-      <x:c r="F37" s="85"/>
-    </x:row>
-    <x:row r="39" ht="36" customHeight="1">
-      <x:c r="A39" s="95" t="str">
+      <x:c r="C38" s="85"/>
+      <x:c r="D38" s="95" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E38" s="84" t="str">
+        <x:v>If approved, request contracts and move the deal to funding</x:v>
+      </x:c>
+      <x:c r="F38" s="85"/>
+    </x:row>
+    <x:row r="40" ht="36" customHeight="1">
+      <x:c r="A40" s="99" t="str">
         <x:v>Disclaimer: All deals are subject to review. Underwriting guidelines, approval criteria, terms and program availability may change from time to time based on market conditions and the complete risk profile of each applicant.</x:v>
       </x:c>
-      <x:c r="B39" s="95"/>
-      <x:c r="C39" s="95"/>
-      <x:c r="D39" s="95"/>
-      <x:c r="E39" s="95"/>
-      <x:c r="F39" s="95"/>
-    </x:row>
-    <x:row r="40" ht="36" customHeight="1">
-      <x:c r="A40" s="95"/>
-      <x:c r="B40" s="95"/>
-      <x:c r="C40" s="95"/>
-      <x:c r="D40" s="95"/>
-      <x:c r="E40" s="95"/>
-      <x:c r="F40" s="95"/>
+      <x:c r="B40" s="99"/>
+      <x:c r="C40" s="99"/>
+      <x:c r="D40" s="99"/>
+      <x:c r="E40" s="99"/>
+      <x:c r="F40" s="99"/>
+    </x:row>
+    <x:row r="41" ht="36" customHeight="1">
+      <x:c r="A41" s="99"/>
+      <x:c r="B41" s="99"/>
+      <x:c r="C41" s="99"/>
+      <x:c r="D41" s="99"/>
+      <x:c r="E41" s="99"/>
+      <x:c r="F41" s="99"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1224,12 +1270,18 @@
     <x:mergeCell ref="B29:F29"/>
     <x:mergeCell ref="B30:F30"/>
     <x:mergeCell ref="B31:F31"/>
-    <x:mergeCell ref="A33:F33"/>
-    <x:mergeCell ref="B34:F34"/>
-    <x:mergeCell ref="B35:F35"/>
-    <x:mergeCell ref="B36:F36"/>
-    <x:mergeCell ref="B37:F37"/>
-    <x:mergeCell ref="A39:F40"/>
+    <x:mergeCell ref="B32:F32"/>
+    <x:mergeCell ref="A34:C34"/>
+    <x:mergeCell ref="D34:F34"/>
+    <x:mergeCell ref="B35:C35"/>
+    <x:mergeCell ref="B36:C36"/>
+    <x:mergeCell ref="B37:C37"/>
+    <x:mergeCell ref="B38:C38"/>
+    <x:mergeCell ref="E35:F35"/>
+    <x:mergeCell ref="E36:F36"/>
+    <x:mergeCell ref="E37:F37"/>
+    <x:mergeCell ref="E38:F38"/>
+    <x:mergeCell ref="A40:F41"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1239,12 +1291,12 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="31" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="25" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="25" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="36" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -1558,19 +1610,19 @@
         <x:v>RESTRICCIONES ESTATALES</x:v>
       </x:c>
       <x:c r="B18" s="70" t="str">
-        <x:v>La mayoría de estados; TX puede usar un préstamo; CA/NY suelen requerir 4 meses bancarios</x:v>
+        <x:v>La mayoría de estados; TX puede usar un préstamo</x:v>
       </x:c>
       <x:c r="C18" s="71" t="str">
         <x:v>La disponibilidad varía; TX/VA pueden exigir más ingresos o antigüedad</x:v>
       </x:c>
       <x:c r="D18" s="72" t="str">
-        <x:v>Algunos programas excluyen VA, CT, UT, ND, AR o TX; verificar antes de enviar</x:v>
+        <x:v>Algunos programas excluyen VA, CT, UT, ND, AR o TX</x:v>
       </x:c>
       <x:c r="E18" s="73" t="str">
         <x:v>Restricciones estatales y de entidad pueden limitar programas especiales</x:v>
       </x:c>
       <x:c r="F18" s="74" t="str">
-        <x:v>Excepciones estatales limitadas; verificar antes de enviar</x:v>
+        <x:v>Excepciones estatales limitadas</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="76" customHeight="1">
@@ -1658,19 +1710,19 @@
         <x:v>CONSIDERACIONES ESPECIALES</x:v>
       </x:c>
       <x:c r="B23" s="70" t="str">
-        <x:v>Mejor valor puede incluir plazos largos, pagos flexibles, mejor precio y opciones de pago anticipado</x:v>
+        <x:v>Descuentos por pago anticipado; plazos largos; pagos flexibles</x:v>
       </x:c>
       <x:c r="C23" s="71" t="str">
-        <x:v>Archivos fuertes pueden lograr mejor plazo, frecuencia, renovación o apoyo de pago</x:v>
+        <x:v>Descuentos por pago anticipado; renovaciones; opciones de liquidación</x:v>
       </x:c>
       <x:c r="D23" s="72" t="str">
-        <x:v>SIC de alto riesgo, defaults satisfechos o posiciones extra pueden evaluarse con factores fuertes</x:v>
+        <x:v>Puede ayudar a crear historial de crédito comercial; acceso a renovaciones</x:v>
       </x:c>
       <x:c r="E23" s="73" t="str">
-        <x:v>Ofertas iniciales, pagos divididos o fondos adicionales pueden existir con factores compensatorios</x:v>
+        <x:v>Financiamiento inicial; puede establecer historial de pagos</x:v>
       </x:c>
       <x:c r="F23" s="74" t="str">
-        <x:v>Solo estructuras especiales, iniciales o de consolidación; montos y plazos más conservadores</x:v>
+        <x:v>Opciones iniciales o de consolidación</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="88" customHeight="1">
@@ -1693,7 +1745,7 @@
         <x:v>Riesgo de fraude financiero; documentos manipulados; stop-payments a funders</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="28" customHeight="1">
+    <x:row r="26" ht="32" customHeight="1">
       <x:c r="A26" s="76" t="str">
         <x:v>POSIBLES EXCEPCIONES Y PUNTOS IMPORTANTES</x:v>
       </x:c>
@@ -1708,7 +1760,7 @@
         <x:v>TÉRMINOS DE APROBACIÓN</x:v>
       </x:c>
       <x:c r="B27" s="84" t="str">
-        <x:v>MONTO, TASA Y PLAZO DEPENDEN DEL PERFIL COMPLETO: INGRESOS, CRÉDITO, DEUDA, ACTIVIDAD BANCARIA E INDUSTRIA.</x:v>
+        <x:v>Monto, tasa y plazo dependen del perfil completo: ingresos, crédito, deuda, actividad bancaria e industria.</x:v>
       </x:c>
       <x:c r="C27" s="84"/>
       <x:c r="D27" s="84"/>
@@ -1720,7 +1772,7 @@
         <x:v>INDUSTRIAS DE ALTO RIESGO</x:v>
       </x:c>
       <x:c r="B28" s="84" t="str">
-        <x:v>SE REVISAN CASO POR CASO; LAS OFERTAS SUELEN SER MENORES, MÁS CORTAS Y CONSERVADORAS.</x:v>
+        <x:v>Se revisan caso por caso; las ofertas suelen ser menores, más cortas y conservadoras.</x:v>
       </x:c>
       <x:c r="C28" s="84"/>
       <x:c r="D28" s="84"/>
@@ -1732,7 +1784,7 @@
         <x:v>CONSOLIDACIÓN</x:v>
       </x:c>
       <x:c r="B29" s="84" t="str">
-        <x:v>SE PERMITEN MÚLTIPLES MCA. PUEDE HABER FONDOS ADICIONALES, REFINANCIAMIENTO O CONSOLIDACIÓN SEGÚN CAPACIDAD.</x:v>
+        <x:v>Se permiten múltiples MCA. Puede haber fondos adicionales, refinanciamiento o consolidación según capacidad.</x:v>
       </x:c>
       <x:c r="C29" s="84"/>
       <x:c r="D29" s="84"/>
@@ -1744,7 +1796,7 @@
         <x:v>ELEGIBILIDAD CON ITIN</x:v>
       </x:c>
       <x:c r="B30" s="84" t="str">
-        <x:v>CASO POR CASO: 12+ MESES OPERANDO Y MÁS DE $25,000 EN INGRESOS MENSUALES.</x:v>
+        <x:v>Caso por caso: 12+ meses operando y más de $25,000 en ingresos mensuales.</x:v>
       </x:c>
       <x:c r="C30" s="84"/>
       <x:c r="D30" s="84"/>
@@ -1756,88 +1808,118 @@
         <x:v>DOCUMENTOS</x:v>
       </x:c>
       <x:c r="B31" s="84" t="str">
-        <x:v>STIPS TÍPICOS: ID, CHEQUE ANULADO, PRUEBA DE PROPIEDAD Y VERIFICACIÓN BANCARIA. OPERACIONES GRANDES PUEDEN REQUERIR IMPUESTOS O ESTADOS FINANCIEROS.</x:v>
+        <x:v>Stips típicos: ID, cheque anulado, prueba de propiedad y verificación bancaria. Operaciones grandes pueden requerir impuestos o estados financieros.</x:v>
       </x:c>
       <x:c r="C31" s="84"/>
       <x:c r="D31" s="84"/>
       <x:c r="E31" s="84"/>
       <x:c r="F31" s="85"/>
     </x:row>
-    <x:row r="33" ht="28" customHeight="1">
-      <x:c r="A33" s="87" t="str">
+    <x:row r="32" ht="62" customHeight="1">
+      <x:c r="A32" s="83" t="str">
+        <x:v>RESPUESTA Y FONDEO</x:v>
+      </x:c>
+      <x:c r="B32" s="84" t="str">
+        <x:v>Las ofertas pueden estar disponibles en 24 horas. El fondeo el mismo día es posible si recibimos rápidamente la información requerida.</x:v>
+      </x:c>
+      <x:c r="C32" s="84"/>
+      <x:c r="D32" s="84"/>
+      <x:c r="E32" s="84"/>
+      <x:c r="F32" s="85"/>
+    </x:row>
+    <x:row r="34" ht="32" customHeight="1">
+      <x:c r="A34" s="87" t="str">
         <x:v>DOCUMENTOS MÍNIMOS REQUERIDOS</x:v>
       </x:c>
-      <x:c r="B33" s="87"/>
-      <x:c r="C33" s="87"/>
-      <x:c r="D33" s="87"/>
-      <x:c r="E33" s="87"/>
-      <x:c r="F33" s="87"/>
-    </x:row>
-    <x:row r="34" ht="44" customHeight="1">
-      <x:c r="A34" s="91" t="n">
+      <x:c r="B34" s="87"/>
+      <x:c r="C34" s="87"/>
+      <x:c r="D34" s="76" t="str">
+        <x:v>PROCESO DE ENVÍO DEL PRÉSTAMO</x:v>
+      </x:c>
+      <x:c r="E34" s="76"/>
+      <x:c r="F34" s="76"/>
+    </x:row>
+    <x:row r="35" ht="58" customHeight="1">
+      <x:c r="A35" s="91" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B34" s="84" t="str">
+      <x:c r="B35" s="84" t="str">
         <x:v>Solicitud firmada</x:v>
       </x:c>
-      <x:c r="C34" s="84"/>
-      <x:c r="D34" s="84"/>
-      <x:c r="E34" s="84"/>
-      <x:c r="F34" s="85"/>
-    </x:row>
-    <x:row r="35" ht="44" customHeight="1">
-      <x:c r="A35" s="91" t="n">
+      <x:c r="C35" s="85"/>
+      <x:c r="D35" s="95" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E35" s="84" t="str">
+        <x:v>Reúna la solicitud firmada y los estados bancarios</x:v>
+      </x:c>
+      <x:c r="F35" s="85"/>
+    </x:row>
+    <x:row r="36" ht="58" customHeight="1">
+      <x:c r="A36" s="91" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B35" s="84" t="str">
+      <x:c r="B36" s="84" t="str">
         <x:v>Últimos 4-6 meses de estados bancarios comerciales completos</x:v>
       </x:c>
-      <x:c r="C35" s="84"/>
-      <x:c r="D35" s="84"/>
-      <x:c r="E35" s="84"/>
-      <x:c r="F35" s="85"/>
-    </x:row>
-    <x:row r="36" ht="54" customHeight="1">
-      <x:c r="A36" s="91" t="n">
+      <x:c r="C36" s="85"/>
+      <x:c r="D36" s="95" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E36" s="84" t="str">
+        <x:v>Envíe el expediente completo a deals@gokapital.com</x:v>
+      </x:c>
+      <x:c r="F36" s="85"/>
+    </x:row>
+    <x:row r="37" ht="66" customHeight="1">
+      <x:c r="A37" s="91" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B36" s="84" t="str">
+      <x:c r="B37" s="84" t="str">
         <x:v>Solicitudes mayores de $150,000: declaraciones de impuestos y estado actual de pérdidas y ganancias</x:v>
       </x:c>
-      <x:c r="C36" s="84"/>
-      <x:c r="D36" s="84"/>
-      <x:c r="E36" s="84"/>
-      <x:c r="F36" s="85"/>
-    </x:row>
-    <x:row r="37" ht="54" customHeight="1">
-      <x:c r="A37" s="91" t="n">
+      <x:c r="C37" s="85"/>
+      <x:c r="D37" s="95" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E37" s="84" t="str">
+        <x:v>Respuesta el mismo día si se recibe antes de la 1:00 p. m.</x:v>
+      </x:c>
+      <x:c r="F37" s="85"/>
+    </x:row>
+    <x:row r="38" ht="66" customHeight="1">
+      <x:c r="A38" s="91" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B37" s="84" t="str">
+      <x:c r="B38" s="84" t="str">
         <x:v>Solicitudes de consolidación: detalles de saldos y cartas de pago</x:v>
       </x:c>
-      <x:c r="C37" s="84"/>
-      <x:c r="D37" s="84"/>
-      <x:c r="E37" s="84"/>
-      <x:c r="F37" s="85"/>
-    </x:row>
-    <x:row r="39" ht="36" customHeight="1">
-      <x:c r="A39" s="95" t="str">
+      <x:c r="C38" s="85"/>
+      <x:c r="D38" s="95" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E38" s="84" t="str">
+        <x:v>Si se aprueba, solicite contratos y pase la operación a fondeo</x:v>
+      </x:c>
+      <x:c r="F38" s="85"/>
+    </x:row>
+    <x:row r="40" ht="36" customHeight="1">
+      <x:c r="A40" s="99" t="str">
         <x:v>Aviso: Todas las operaciones están sujetas a revisión. Las guías de suscripción, los criterios de aprobación, los términos y la disponibilidad de los programas pueden cambiar según las condiciones del mercado y el perfil de riesgo completo de cada solicitante.</x:v>
       </x:c>
-      <x:c r="B39" s="95"/>
-      <x:c r="C39" s="95"/>
-      <x:c r="D39" s="95"/>
-      <x:c r="E39" s="95"/>
-      <x:c r="F39" s="95"/>
-    </x:row>
-    <x:row r="40" ht="36" customHeight="1">
-      <x:c r="A40" s="95"/>
-      <x:c r="B40" s="95"/>
-      <x:c r="C40" s="95"/>
-      <x:c r="D40" s="95"/>
-      <x:c r="E40" s="95"/>
-      <x:c r="F40" s="95"/>
+      <x:c r="B40" s="99"/>
+      <x:c r="C40" s="99"/>
+      <x:c r="D40" s="99"/>
+      <x:c r="E40" s="99"/>
+      <x:c r="F40" s="99"/>
+    </x:row>
+    <x:row r="41" ht="36" customHeight="1">
+      <x:c r="A41" s="99"/>
+      <x:c r="B41" s="99"/>
+      <x:c r="C41" s="99"/>
+      <x:c r="D41" s="99"/>
+      <x:c r="E41" s="99"/>
+      <x:c r="F41" s="99"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1849,12 +1931,18 @@
     <x:mergeCell ref="B29:F29"/>
     <x:mergeCell ref="B30:F30"/>
     <x:mergeCell ref="B31:F31"/>
-    <x:mergeCell ref="A33:F33"/>
-    <x:mergeCell ref="B34:F34"/>
-    <x:mergeCell ref="B35:F35"/>
-    <x:mergeCell ref="B36:F36"/>
-    <x:mergeCell ref="B37:F37"/>
-    <x:mergeCell ref="A39:F40"/>
+    <x:mergeCell ref="B32:F32"/>
+    <x:mergeCell ref="A34:C34"/>
+    <x:mergeCell ref="D34:F34"/>
+    <x:mergeCell ref="B35:C35"/>
+    <x:mergeCell ref="B36:C36"/>
+    <x:mergeCell ref="B37:C37"/>
+    <x:mergeCell ref="B38:C38"/>
+    <x:mergeCell ref="E35:F35"/>
+    <x:mergeCell ref="E36:F36"/>
+    <x:mergeCell ref="E37:F37"/>
+    <x:mergeCell ref="E38:F38"/>
+    <x:mergeCell ref="A40:F41"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>